<commit_message>
Make configured celestial surface rotation coherent and readable
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/planet.xlsx
+++ b/space-battleship/config_excel/planet.xlsx
@@ -1371,8 +1371,10 @@
       <ns0:c r="E5">
         <ns0:v>150</ns0:v>
       </ns0:c>
-      <ns0:c r="G5" t="str">
-        <ns0:v>{"surfaceTexture":"res://assets/planets/t587e_surface.png","cloudTexture":"res://assets/planets/t587e_surface.png","radiusScale":1.05,"axisRatio":0.93,"surfaceSpeed":0.0017,"cloudSpeed":0.0022,"cloudOpacity":0.12,"shadowStrength":0.53,"glowStrength":0.38,"atmosphereColor":"e8d3a2","coronaWidth":0.035}</ns0:v>
+      <ns0:c r="G5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>{"surfaceTexture":"res://assets/planets/t587e_surface.png","cloudTexture":"res://assets/planets/t587e_surface.png","radiusScale":1.05,"axisRatio":0.93,"surfaceSpeed":0.006,"cloudSpeed":0.0075,"cloudOpacity":0.12,"shadowStrength":0.53,"glowStrength":0.38,"atmosphereColor":"e8d3a2","coronaWidth":0.035}</ns0:t>
+        </ns0:is>
       </ns0:c>
       <ns0:c r="H5" t="n">
         <ns0:v>10</ns0:v>
@@ -1397,8 +1399,10 @@
       <ns0:c r="E6">
         <ns0:v>200</ns0:v>
       </ns0:c>
-      <ns0:c r="G6" t="str">
-        <ns0:v>{"surfaceTexture":"res://assets/planets/stellar_plasma.png","cloudOpacity":0,"shadowStrength":0,"emission":1.3,"radiusScale":0.83,"detailScale":3.2,"detailStrength":0.7,"surfaceSpeed":0.002,"cloudSpeed":0.0028,"surfaceTint":"fff4c9","shadowTint":"d49642","atmosphereColor":"ffdda0","coronaWidth":0.085,"glowStrength":0.56,"flareStrength":0.12}</ns0:v>
+      <ns0:c r="G6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>{"surfaceTexture":"res://assets/planets/stellar_plasma.png","cloudOpacity":0,"shadowStrength":0,"emission":1.3,"radiusScale":0.83,"detailScale":1.2,"detailStrength":0.9,"surfaceSpeed":0.0065,"cloudSpeed":0.008,"surfaceTint":"fff4c9","shadowTint":"d49642","atmosphereColor":"ffdda0","coronaWidth":0.085,"glowStrength":0.56,"flareStrength":0.12}</ns0:t>
+        </ns0:is>
       </ns0:c>
       <ns0:c r="H6" t="n">
         <ns0:v>15</ns0:v>
@@ -1423,8 +1427,10 @@
       <ns0:c r="E7">
         <ns0:v>250</ns0:v>
       </ns0:c>
-      <ns0:c r="G7" t="str">
-        <ns0:v>{"surfaceTexture":"res://assets/planets/stellar_plasma.png","cloudOpacity":0,"shadowStrength":0,"emission":1.1,"radiusScale":1.22,"detailScale":0.55,"detailStrength":1,"surfaceSpeed":0.0007,"cloudSpeed":0.0011,"surfaceTint":"ff8539","shadowTint":"6b100c","atmosphereColor":"ee6333","coronaWidth":0.2,"glowStrength":0.27,"pulseStrength":0.009,"pulseSpeed":0.05}</ns0:v>
+      <ns0:c r="G7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>{"surfaceTexture":"res://assets/planets/stellar_plasma.png","cloudOpacity":0,"shadowStrength":0,"emission":1.1,"radiusScale":1.22,"detailScale":0.55,"detailStrength":1,"surfaceSpeed":0.0035,"cloudSpeed":0.0045,"surfaceTint":"ff8539","shadowTint":"6b100c","atmosphereColor":"ee6333","coronaWidth":0.2,"glowStrength":0.27,"pulseStrength":0.009,"pulseSpeed":0.05}</ns0:t>
+        </ns0:is>
       </ns0:c>
       <ns0:c r="H7" t="n">
         <ns0:v>20</ns0:v>
@@ -1449,8 +1455,10 @@
       <ns0:c r="E8">
         <ns0:v>300</ns0:v>
       </ns0:c>
-      <ns0:c r="G8" t="str">
-        <ns0:v>{"surfaceTexture":"res://assets/planets/stellar_plasma.png","cloudOpacity":0,"shadowStrength":0,"emission":1.6,"radiusScale":0.22,"detailScale":2,"detailStrength":0.06,"surfaceSpeed":0.006,"cloudSpeed":0.009,"surfaceTint":"f6ffff","shadowTint":"a0d9ff","atmosphereColor":"96ceff","coronaWidth":0.065,"glowStrength":0.8}</ns0:v>
+      <ns0:c r="G8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>{"surfaceTexture":"res://assets/planets/stellar_plasma.png","cloudOpacity":0,"shadowStrength":0,"emission":1.6,"radiusScale":0.22,"detailScale":1.0,"detailStrength":0.8,"surfaceSpeed":0.008,"cloudSpeed":0.01,"surfaceTint":"f6ffff","shadowTint":"a0d9ff","atmosphereColor":"96ceff","coronaWidth":0.065,"glowStrength":0.8}</ns0:t>
+        </ns0:is>
       </ns0:c>
       <ns0:c r="H8" t="n">
         <ns0:v>25</ns0:v>
@@ -1475,8 +1483,10 @@
       <ns0:c r="E9">
         <ns0:v>350</ns0:v>
       </ns0:c>
-      <ns0:c r="G9" t="str">
-        <ns0:v>{"surfaceTexture":"res://assets/planets/stellar_plasma.png","cloudOpacity":0,"shadowStrength":0,"emission":1.7,"radiusScale":0.16,"detailStrength":0.12,"surfaceSpeed":0.35,"cloudSpeed":0.42,"surfaceTint":"edffff","shadowTint":"8bc9ff","atmosphereColor":"6fbfff","coronaWidth":0.12,"glowStrength":0.8,"beamLength":7.5,"beamWidth":0.2,"beamSpeed":1.6,"magnetosphere":0.55}</ns0:v>
+      <ns0:c r="G9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>{"surfaceTexture":"res://assets/planets/stellar_plasma.png","cloudOpacity":0,"shadowStrength":0,"emission":1.7,"radiusScale":0.16,"detailStrength":0.85,"surfaceSpeed":0.02,"cloudSpeed":0.025,"surfaceTint":"edffff","shadowTint":"8bc9ff","atmosphereColor":"6fbfff","coronaWidth":0.12,"glowStrength":0.8,"beamLength":7.5,"beamWidth":0.2,"beamSpeed":1.6,"magnetosphere":0.55,"detailScale":1.0}</ns0:t>
+        </ns0:is>
       </ns0:c>
       <ns0:c r="H9" t="n">
         <ns0:v>30</ns0:v>

</xml_diff>